<commit_message>
Ch281: PDF regeneres 8 poles + fiche/data book/zip aux bons noms
</commit_message>
<xml_diff>
--- a/Data_Book_EnerTchad.xlsx
+++ b/Data_Book_EnerTchad.xlsx
@@ -144,13 +144,13 @@
     <t xml:space="preserve">Poles chaine (4)</t>
   </si>
   <si>
-    <t xml:space="preserve">Amont · Intermediaire · Aval · EnerChimie</t>
+    <t xml:space="preserve">Amont · Intermediaire · Aval · Petrochimie</t>
   </si>
   <si>
     <t xml:space="preserve">Poles supports (4)</t>
   </si>
   <si>
-    <t xml:space="preserve">GreenTech · EnerTech · EnerTalents · EnerConseils</t>
+    <t xml:space="preserve">GreenTech · TchadiTech · Tchaditude · EnerConseils</t>
   </si>
   <si>
     <t xml:space="preserve">Signature</t>
@@ -681,20 +681,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -718,19 +722,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -989,73 +993,73 @@
   <dimension ref="A1:A15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="110"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1078,231 +1082,231 @@
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="E2" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="E3" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="E4" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="E5" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="E6" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="E7" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="E8" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="E9" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="E10" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="E11" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="E12" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="7" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1325,211 +1329,211 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="F2" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="F3" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="F4" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="F5" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="F6" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="F7" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="F8" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="F9" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1552,231 +1556,231 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="F3" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="F4" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+    <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>119</v>
       </c>
     </row>
@@ -1799,100 +1803,100 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="C2" s="8" t="n">
         <v>0.35</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="9" t="n">
         <v>0.25</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="8" t="n">
         <v>0.15</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="9" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
         <v>0.08</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="9" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="11" t="n">
+      <c r="B8" s="11"/>
+      <c r="C8" s="12" t="n">
         <f aca="false">SUM(C2:C7)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
         <v>136</v>
       </c>
     </row>
@@ -1915,171 +1919,171 @@
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="7" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="F4" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="F5" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="F6" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>165</v>
       </c>
     </row>

</xml_diff>